<commit_message>
EPBDS-16318 Draw the data model as an ER diagram of typed entities
A vocabulary reported no values at all, so a client could only render it as an
empty datatype, and a datatype was a named dot whose fields lived in the side
panel. A datatype node now carries the values a vocabulary declares — typed, in
declaration order, previewed by its first and last ones — and the graph screen
draws every datatype as an entity box listing its fields or its values.
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.webstudio/test-resources/org/openl/studio/projects/service/tables/graph/DataModel/DataModel.xlsx
+++ b/STUDIO/org.openl.rules.webstudio/test-resources/org/openl/studio/projects/service/tables/graph/DataModel/DataModel.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C24"/>
+  <dimension ref="B1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -422,6 +422,11 @@
           <t>Datatype Vehicle</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Datatype Score &lt;Integer&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -434,6 +439,9 @@
           <t>make</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -446,6 +454,14 @@
           <t>year</t>
         </is>
       </c>
+      <c r="E3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="E4" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -453,6 +469,9 @@
           <t>Datatype Car extends Vehicle</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>400</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -465,6 +484,14 @@
           <t>model</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7" t="n">
+        <v>600</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -472,6 +499,9 @@
           <t>Datatype Driver</t>
         </is>
       </c>
+      <c r="E8" t="n">
+        <v>700</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
@@ -484,6 +514,9 @@
           <t>name</t>
         </is>
       </c>
+      <c r="E9" t="n">
+        <v>800</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
@@ -494,6 +527,13 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>mentor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Datatype Blank &lt;String&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>